<commit_message>
Redesign CME expectations workbook
</commit_message>
<xml_diff>
--- a/files/BUS331_InvProject_CMEMatrix_Template.xlsx
+++ b/files/BUS331_InvProject_CMEMatrix_Template.xlsx
@@ -660,7 +660,8 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="151" uniqueCount="79">
   <si>
-    <t>BUS 331 — CME Matrix Template  |  Phase 3: The Bridge</t>
+    <t>BUS 331 — CME Matrix Template
+Phase 2 — Workstream A: Capital Market Expectations</t>
   </si>
   <si>
     <t>Capital Market Expectations Matrix  |  Endicott College</t>
@@ -687,7 +688,7 @@
     <t>Step 4 — Enter IPS constraints</t>
   </si>
   <si>
-    <t>In Section 5 of each tab, enter each client's maximum σ limit and maximum drawdown (Tripwire) from your Phase 2 IPS. The Status column will flag any constraint violations.</t>
+    <t>Use the Phase 1 IPS constraints. In Section 5 of each tab, enter each client's maximum σ limit and maximum drawdown (Tripwire). The Status column will flag any constraint violations.</t>
   </si>
   <si>
     <t>Step 5 — Run Excel Solver</t>
@@ -732,7 +733,7 @@
     <t>Capital Market Expectations Matrix  —  Base Case</t>
   </si>
   <si>
-    <t>BUS 331 Investments  |  Endicott College  |  Phase 3: The Bridge</t>
+    <t>BUS 331 Investments  |  Endicott College  |  Phase 2 — Workstream A: Capital Market Expectations</t>
   </si>
   <si>
     <t>⚠  All expected return and standard deviation inputs must be sourced from your Phase 1 macro thesis and verified against FactSet / FRED.</t>
@@ -829,11 +830,11 @@
     <t>SECTION 5 — IPS CONSTRAINT CHECK</t>
   </si>
   <si>
-    <t>After entering weights, verify each client's portfolio σ does not exceed their IPS standard deviation limit from Phase 2. Enter the IPS limit below for reference.</t>
+    <t>Use the Phase 1 IPS constraints. After entering weights, verify each client's portfolio σ does not exceed the approved standard deviation limit. Enter the IPS limits below for reference.</t>
   </si>
   <si>
     <t>IPS Max σ
-(from Phase 2)</t>
+(Phase 1 IPS)</t>
   </si>
   <si>
     <t>Portfolio σ
@@ -1237,7 +1238,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="19" fillId="9" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -1331,6 +1332,9 @@
     </xf>
     <xf numFmtId="0" fontId="18" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1695,129 +1699,178 @@
       <c r="B3" s="13"/>
       <c r="C3" s="13"/>
     </row>
-    <row r="5" spans="1:3" ht="13.5" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="5" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B5" s="12" t="inlineStr">
+        <is>
+          <t>This workbook sets the strategic allocation inputs that support the Phase 2 client portfolios and stress testing.</t>
+        </is>
+      </c>
+      <c r="C5" s="12"/>
+    </row>
     <row r="6" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B6" s="15" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B7" s="12" t="s">
-        <v>3</v>
+      <c r="B6" s="15" t="inlineStr">
+        <is>
+          <t>Step 1 — Macro view</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" spans="1:9" ht="34" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B7" s="12" t="inlineStr">
+        <is>
+          <t>Finalize the Phase 1 economic story: growth, inflation, rates, and the key downside risk. These judgments anchor every assumption that follows.</t>
+        </is>
       </c>
       <c r="C7" s="12"/>
     </row>
     <row r="8" spans="1:3" ht="13.5" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="9" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B9" s="15" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B10" s="12" t="s">
-        <v>5</v>
+      <c r="B9" s="15" t="inlineStr">
+        <is>
+          <t>Step 2 — Build expectations</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" spans="1:9" ht="34" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B10" s="12" t="inlineStr">
+        <is>
+          <t>On BASE CASE, enter expected return, volatility, one source with its as-of date, a one-sentence macro rationale, and the specific Bear Case change you expect for each asset class.</t>
+        </is>
       </c>
       <c r="C10" s="12"/>
     </row>
     <row r="11" spans="1:3" ht="13.5" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="12" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B12" s="15" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B13" s="12" t="s">
-        <v>7</v>
+      <c r="B12" s="15" t="inlineStr">
+        <is>
+          <t>Step 3 — Build Base and Bear scenarios</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" spans="1:9" ht="34" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B13" s="12" t="inlineStr">
+        <is>
+          <t>Complete both scenarios. Change only returns, volatility, or correlations supported by the downside story; do not mechanically lower every return or push every correlation upward.</t>
+        </is>
       </c>
       <c r="C13" s="12"/>
     </row>
     <row r="14" spans="1:3" ht="13.5" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="15" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B15" s="15" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B16" s="12" t="s">
-        <v>9</v>
+      <c r="B15" s="15" t="inlineStr">
+        <is>
+          <t>Step 4 — Apply client constraints</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" spans="1:9" ht="34" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B16" s="12" t="inlineStr">
+        <is>
+          <t>Use the Phase 1 IPS constraints. Enter each client's maximum portfolio σ and drawdown tripwire in Section 5 of both scenario sheets.</t>
+        </is>
       </c>
       <c r="C16" s="12"/>
     </row>
     <row r="17" spans="2:3" ht="13.5" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="18" spans="2:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B18" s="15" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="19" spans="2:3" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B19" s="12" t="s">
-        <v>11</v>
+      <c r="B18" s="15" t="inlineStr">
+        <is>
+          <t>Step 5 — Run Solver-supported allocation</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" spans="1:9" ht="34" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B19" s="12" t="inlineStr">
+        <is>
+          <t>Run Solver one client at a time using the numbered checklist on that scenario sheet. Solver supports the allocation decision; it does not replace judgment.</t>
+        </is>
       </c>
       <c r="C19" s="12"/>
     </row>
     <row r="20" spans="2:3" ht="13.5" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="21" spans="2:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B21" s="15" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="22" spans="2:3" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B22" s="12" t="s">
-        <v>13</v>
+      <c r="B21" s="15" t="inlineStr">
+        <is>
+          <t>Step 6 — Stress test and compare</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" spans="1:9" ht="34" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B22" s="12" t="inlineStr">
+        <is>
+          <t>Compare Base and Bear results, constraint status, concentration, and trade-offs. Use the Bear Case to test resilience—not to manufacture a uniformly worse forecast.</t>
+        </is>
       </c>
       <c r="C22" s="12"/>
     </row>
     <row r="23" spans="2:3" ht="13.5" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="24" spans="2:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B24" s="15" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="25" spans="2:3" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B25" s="12" t="s">
-        <v>15</v>
+      <c r="B24" s="15" t="inlineStr">
+        <is>
+          <t>Step 7 — Recommend and document</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" spans="1:9" ht="34" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B25" s="12" t="inlineStr">
+        <is>
+          <t>Complete each client's Read the Result prompts, choose a defensible recommendation, and record any AI-assisted inputs in the team's AI Audit Log with independent verification.</t>
+        </is>
       </c>
       <c r="C25" s="12"/>
     </row>
     <row r="27" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B27" s="11" t="s">
-        <v>16</v>
+      <c r="B27" s="11" t="inlineStr">
+        <is>
+          <t>WORKFLOW AT A GLANCE</t>
+        </is>
       </c>
       <c r="C27" s="11"/>
     </row>
-    <row r="28" spans="2:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B28" s="10" t="s">
-        <v>17</v>
+    <row r="28" spans="1:9" ht="26" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B28" s="10" t="inlineStr">
+        <is>
+          <t>Macro view → expectations → Base/Bear scenarios → client constraints</t>
+        </is>
       </c>
       <c r="C28" s="10"/>
     </row>
-    <row r="29" spans="2:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B29" s="10" t="s">
-        <v>18</v>
+    <row r="29" spans="1:9" ht="26" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B29" s="10" t="inlineStr">
+        <is>
+          <t>Solver-supported allocation → stress test → recommendation</t>
+        </is>
       </c>
       <c r="C29" s="10"/>
     </row>
-    <row r="30" spans="2:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B30" s="10" t="s">
-        <v>19</v>
+    <row r="30" spans="1:9" ht="26" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B30" s="10" t="inlineStr">
+        <is>
+          <t>Use the full Solver checklist and Read the Result prompts on each scenario sheet.</t>
+        </is>
       </c>
       <c r="C30" s="10"/>
     </row>
-    <row r="31" spans="2:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B31" s="10" t="s">
-        <v>20</v>
+    <row r="31" spans="1:9" ht="26" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B31" s="10" t="inlineStr">
+        <is>
+          <t>Keep assumptions sourced, dated, and tied to the team's economic story.</t>
+        </is>
       </c>
       <c r="C31" s="10"/>
     </row>
-    <row r="32" spans="2:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B32" s="10" t="s">
-        <v>21</v>
+    <row r="32" spans="1:9" ht="26" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B32" s="10" t="inlineStr">
+        <is>
+          <t>A mathematically optimal result is not automatically a suitable client recommendation.</t>
+        </is>
       </c>
       <c r="C32" s="10"/>
     </row>
-    <row r="33" spans="2:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B33" s="10" t="s">
-        <v>22</v>
+    <row r="33" spans="1:9" ht="26" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B33" s="10" t="inlineStr">
+        <is>
+          <t>Document consequential judgment and any AI-assisted input in the project audit trail.</t>
+        </is>
       </c>
       <c r="C33" s="10"/>
     </row>
@@ -1850,14 +1903,16 @@
   <sheetPr>
     <tabColor rgb="FF1F6B3A"/>
   </sheetPr>
-  <dimension ref="A1:I69"/>
+  <dimension ref="A1:I74"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="2" customWidth="1"/>
-    <col min="2" max="2" width="26" customWidth="1"/>
-    <col min="3" max="5" width="18" customWidth="1"/>
-    <col min="6" max="8" width="20" customWidth="1"/>
-    <col min="9" max="9" width="29.5703125" customWidth="1"/>
+    <col min="2" max="2" width="22" customWidth="1"/>
+    <col min="3" max="4" width="14" customWidth="1"/>
+    <col min="5" max="5" width="18" customWidth="1"/>
+    <col min="6" max="6" width="13" customWidth="1"/>
+    <col min="7" max="8" width="18" customWidth="1"/>
+    <col min="9" max="9" width="27" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -1887,9 +1942,11 @@
       <c r="H3" s="8"/>
       <c r="I3" s="8"/>
     </row>
-    <row r="4" spans="1:9" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="7" t="s">
-        <v>25</v>
+    <row r="4" spans="1:9" ht="38" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>⚠  Build each expectation from the Phase 1 macro view, one dated source, and a concise economic rationale. Plan the specific Bear Case change before optimizing.</t>
+        </is>
       </c>
       <c r="B4" s="7"/>
       <c r="C4" s="7"/>
@@ -1902,8 +1959,10 @@
     </row>
     <row r="5" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="6" spans="1:9" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="6" t="s">
-        <v>26</v>
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>SECTION 1 — EXPECTATION BUILDER</t>
+        </is>
       </c>
       <c r="B6" s="6"/>
       <c r="C6" s="6"/>
@@ -1914,24 +1973,43 @@
       <c r="H6" s="6"/>
       <c r="I6" s="6"/>
     </row>
-    <row r="7" spans="1:9" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B7" s="16" t="s">
-        <v>27</v>
-      </c>
-      <c r="C7" s="16" t="s">
-        <v>28</v>
-      </c>
-      <c r="D7" s="16" t="s">
-        <v>29</v>
-      </c>
-      <c r="E7" s="5" t="s">
-        <v>30</v>
+    <row r="7" spans="1:9" ht="42" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B7" s="16" t="inlineStr">
+        <is>
+          <t>Asset Class</t>
+        </is>
+      </c>
+      <c r="C7" s="16" t="inlineStr">
+        <is>
+          <t>Expected Return
+E(R)</t>
+        </is>
+      </c>
+      <c r="D7" s="16" t="inlineStr">
+        <is>
+          <t>Volatility
+(σ)</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>Source + as-of date</t>
+        </is>
       </c>
       <c r="F7" s="5"/>
-      <c r="G7" s="5"/>
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>One-sentence macro rationale</t>
+        </is>
+      </c>
       <c r="H7" s="5"/>
-    </row>
-    <row r="8" spans="1:9" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I7" t="inlineStr" s="16">
+        <is>
+          <t>Bear-case change &amp; why</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" spans="1:9" ht="50" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B8" s="17" t="s">
         <v>31</v>
       </c>
@@ -1941,8 +2019,9 @@
       <c r="F8" s="4"/>
       <c r="G8" s="4"/>
       <c r="H8" s="4"/>
-    </row>
-    <row r="9" spans="1:9" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I8" s="4"/>
+    </row>
+    <row r="9" spans="1:9" ht="50" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B9" s="17" t="s">
         <v>32</v>
       </c>
@@ -1952,8 +2031,9 @@
       <c r="F9" s="4"/>
       <c r="G9" s="4"/>
       <c r="H9" s="4"/>
-    </row>
-    <row r="10" spans="1:9" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I9" s="4"/>
+    </row>
+    <row r="10" spans="1:9" ht="50" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B10" s="17" t="s">
         <v>33</v>
       </c>
@@ -1963,6 +2043,7 @@
       <c r="F10" s="4"/>
       <c r="G10" s="4"/>
       <c r="H10" s="4"/>
+      <c r="I10" s="4"/>
     </row>
     <row r="11" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="12" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -1979,9 +2060,11 @@
       <c r="H13" s="11"/>
       <c r="I13" s="11"/>
     </row>
-    <row r="14" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="12" t="s">
-        <v>35</v>
+    <row r="14" spans="1:9" ht="32" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="12" t="inlineStr">
+        <is>
+          <t>Enter pairwise correlations (–1.0 to 1.0). Diagonal = 1.00. Keep them consistent with the same Base Case story.</t>
+        </is>
       </c>
       <c r="B14" s="12"/>
       <c r="C14" s="12"/>
@@ -2060,9 +2143,11 @@
       <c r="H21" s="11"/>
       <c r="I21" s="11"/>
     </row>
-    <row r="22" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="12" t="s">
-        <v>39</v>
+    <row r="22" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="12" t="inlineStr">
+        <is>
+          <t>Enter each client's starting weights, then run Solver one client at a time. Keep the Solver-supported weights only after completing the Section 6 usability checks.</t>
+        </is>
       </c>
       <c r="B22" s="12"/>
       <c r="C22" s="12"/>
@@ -2212,9 +2297,11 @@
       <c r="H34" s="11"/>
       <c r="I34" s="11"/>
     </row>
-    <row r="35" spans="1:9" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="12" t="s">
-        <v>54</v>
+    <row r="35" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="12" t="inlineStr">
+        <is>
+          <t>Use the Phase 1 IPS constraints. Portfolio σ is the active Solver risk limit; the drawdown tripwire remains a separate stress-test and recommendation check.</t>
+        </is>
       </c>
       <c r="B35" s="12"/>
       <c r="C35" s="12"/>
@@ -2433,22 +2520,269 @@
       <c r="H54" s="3"/>
     </row>
     <row r="55" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="56" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="57" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="58" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="59" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="60" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="61" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="62" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="63" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="64" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="65" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="56" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A56" t="inlineStr" s="11">
+        <is>
+          <t>SECTION 6 — SOLVER SETUP — RUN ONE CLIENT AT A TIME</t>
+        </is>
+      </c>
+      <c r="B56" s="11"/>
+      <c r="C56" s="11"/>
+      <c r="D56" s="11"/>
+      <c r="E56" s="11"/>
+      <c r="F56" s="11"/>
+      <c r="G56" s="11"/>
+      <c r="H56" s="11"/>
+      <c r="I56" s="11"/>
+    </row>
+    <row r="57" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A57" t="inlineStr" s="12">
+        <is>
+          <t>Use this checklist on the Base Case sheet. Solver supports the recommendation; it does not decide whether the result fits the client.</t>
+        </is>
+      </c>
+      <c r="B57" s="12"/>
+      <c r="C57" s="12"/>
+      <c r="D57" s="12"/>
+      <c r="E57" s="12"/>
+      <c r="F57" s="12"/>
+      <c r="G57" s="12"/>
+      <c r="H57" s="12"/>
+      <c r="I57" s="12"/>
+    </row>
+    <row r="58" spans="1:9" ht="34" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B58" t="inlineStr" s="12">
+        <is>
+          <t>1. Understand the task — Solver searches the three asset-class weights for one client and scenario to maximize that row's Sharpe Ratio while respecting the listed constraints.</t>
+        </is>
+      </c>
+      <c r="C58" s="12"/>
+      <c r="D58" s="12"/>
+      <c r="E58" s="12"/>
+      <c r="F58" s="12"/>
+      <c r="G58" s="12"/>
+      <c r="H58" s="12"/>
+      <c r="I58" s="12"/>
+    </row>
+    <row r="59" spans="1:9" ht="34" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B59" t="inlineStr" s="12">
+        <is>
+          <t>2. Select the objective — Set I24, I25, or I26 to Max for Client 1, 2, or 3. Work on one client row at a time.</t>
+        </is>
+      </c>
+      <c r="C59" s="12"/>
+      <c r="D59" s="12"/>
+      <c r="E59" s="12"/>
+      <c r="F59" s="12"/>
+      <c r="G59" s="12"/>
+      <c r="H59" s="12"/>
+      <c r="I59" s="12"/>
+    </row>
+    <row r="60" spans="1:9" ht="34" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B60" t="inlineStr" s="12">
+        <is>
+          <t>3. Select changing cells — Use C24:E24, C25:E25, or C26:E26 for the same client row. These are the U.S. equity, fixed-income, and cash weights.</t>
+        </is>
+      </c>
+      <c r="C60" s="12"/>
+      <c r="D60" s="12"/>
+      <c r="E60" s="12"/>
+      <c r="F60" s="12"/>
+      <c r="G60" s="12"/>
+      <c r="H60" s="12"/>
+      <c r="I60" s="12"/>
+    </row>
+    <row r="61" spans="1:9" ht="42" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B61" t="inlineStr" s="32">
+        <is>
+          <t>4. Add the actual constraints — Matching row F = 1; matching row C:E ≥ 0; and H24 ≤ C37, H25 ≤ C38, or H26 ≤ C39. Drawdown in E37:E39 is not calculated by this model and is not a Solver constraint.</t>
+        </is>
+      </c>
+      <c r="C61" s="32"/>
+      <c r="D61" s="32"/>
+      <c r="E61" s="32"/>
+      <c r="F61" s="32"/>
+      <c r="G61" s="32"/>
+      <c r="H61" s="32"/>
+      <c r="I61" s="32"/>
+    </row>
+    <row r="62" spans="1:9" ht="34" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B62" t="inlineStr" s="12">
+        <is>
+          <t>5. Run Solver — Choose GRG Nonlinear, click Solve, and keep the Solver solution only if Solver reports a solution and the next checks pass.</t>
+        </is>
+      </c>
+      <c r="C62" s="12"/>
+      <c r="D62" s="12"/>
+      <c r="E62" s="12"/>
+      <c r="F62" s="12"/>
+      <c r="G62" s="12"/>
+      <c r="H62" s="12"/>
+      <c r="I62" s="12"/>
+    </row>
+    <row r="63" spans="1:9" ht="42" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B63" t="inlineStr" s="12">
+        <is>
+          <t>6. Confirm it is usable — Weights are nonnegative and total 100%; portfolio σ is within the matching Phase 1 limit; Status shows PASS; inputs use consistent percentage units; and the allocation is economically plausible for the client.</t>
+        </is>
+      </c>
+      <c r="C63" s="12"/>
+      <c r="D63" s="12"/>
+      <c r="E63" s="12"/>
+      <c r="F63" s="12"/>
+      <c r="G63" s="12"/>
+      <c r="H63" s="12"/>
+      <c r="I63" s="12"/>
+    </row>
+    <row r="64" spans="1:9" ht="42" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B64" t="inlineStr" s="32">
+        <is>
+          <t>7. If Solver is infeasible — Check the objective/changing/constraint cells all use the same client row, correlations are between –1 and 1, percentages were entered as percentages, and the IPS σ limit is entered. Do not relax an approved IPS limit to force a solution.</t>
+        </is>
+      </c>
+      <c r="C64" s="32"/>
+      <c r="D64" s="32"/>
+      <c r="E64" s="32"/>
+      <c r="F64" s="32"/>
+      <c r="G64" s="32"/>
+      <c r="H64" s="32"/>
+      <c r="I64" s="32"/>
+    </row>
+    <row r="65" ht="42" customHeight="1" x14ac:dyDescent="0.25" spans="1:9">
+      <c r="B65" t="inlineStr" s="32">
+        <is>
+          <t>8. If the allocation looks implausible — Recheck return, volatility, correlation, source/date, and starting weights. The Sharpe objective can concentrate a portfolio; use the stress test and client mandate before recommending it.</t>
+        </is>
+      </c>
+      <c r="C65" s="32"/>
+      <c r="D65" s="32"/>
+      <c r="E65" s="32"/>
+      <c r="F65" s="32"/>
+      <c r="G65" s="32"/>
+      <c r="H65" s="32"/>
+      <c r="I65" s="32"/>
+    </row>
     <row r="66" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="67" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="68" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="69" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="68" ht="24" customHeight="1" x14ac:dyDescent="0.25" spans="1:9">
+      <c r="A68" t="inlineStr" s="11">
+        <is>
+          <t>SECTION 7 — READ THE RESULT</t>
+        </is>
+      </c>
+      <c r="B68" s="11"/>
+      <c r="C68" s="11"/>
+      <c r="D68" s="11"/>
+      <c r="E68" s="11"/>
+      <c r="F68" s="11"/>
+      <c r="G68" s="11"/>
+      <c r="H68" s="11"/>
+      <c r="I68" s="11"/>
+    </row>
+    <row r="69" ht="30" customHeight="1" x14ac:dyDescent="0.25" spans="1:9">
+      <c r="A69" t="inlineStr" s="12">
+        <is>
+          <t>After Solver, interpret each client's result against the starting allocation. Keep answers concise and decision-focused.</t>
+        </is>
+      </c>
+      <c r="B69" s="12"/>
+      <c r="C69" s="12"/>
+      <c r="D69" s="12"/>
+      <c r="E69" s="12"/>
+      <c r="F69" s="12"/>
+      <c r="G69" s="12"/>
+      <c r="H69" s="12"/>
+      <c r="I69" s="12"/>
+    </row>
+    <row r="70" spans="1:9" ht="38" customHeight="1">
+      <c r="B70" t="inlineStr" s="16">
+        <is>
+          <t>Client</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr" s="16">
+        <is>
+          <t>Change from starting allocation</t>
+        </is>
+      </c>
+      <c r="D70" s="16"/>
+      <c r="E70" t="inlineStr" s="16">
+        <is>
+          <t>Assumption or constraint driving it</t>
+        </is>
+      </c>
+      <c r="F70" s="16"/>
+      <c r="G70" t="inlineStr" s="16">
+        <is>
+          <t>Main trade-off</t>
+        </is>
+      </c>
+      <c r="H70" s="16"/>
+      <c r="I70" t="inlineStr" s="16">
+        <is>
+          <t>Revisit trigger</t>
+        </is>
+      </c>
+    </row>
+    <row r="71" spans="1:9" ht="52" customHeight="1">
+      <c r="B71" t="inlineStr" s="17">
+        <is>
+          <t>Client 1</t>
+        </is>
+      </c>
+      <c r="C71" s="4"/>
+      <c r="D71" s="4"/>
+      <c r="E71" s="4"/>
+      <c r="F71" s="4"/>
+      <c r="G71" s="4"/>
+      <c r="H71" s="4"/>
+      <c r="I71" s="4"/>
+    </row>
+    <row r="72" spans="1:9" ht="52" customHeight="1">
+      <c r="B72" t="inlineStr" s="17">
+        <is>
+          <t>Client 2</t>
+        </is>
+      </c>
+      <c r="C72" s="4"/>
+      <c r="D72" s="4"/>
+      <c r="E72" s="4"/>
+      <c r="F72" s="4"/>
+      <c r="G72" s="4"/>
+      <c r="H72" s="4"/>
+      <c r="I72" s="4"/>
+    </row>
+    <row r="73" spans="1:9" ht="52" customHeight="1">
+      <c r="B73" t="inlineStr" s="17">
+        <is>
+          <t>Client 3</t>
+        </is>
+      </c>
+      <c r="C73" s="4"/>
+      <c r="D73" s="4"/>
+      <c r="E73" s="4"/>
+      <c r="F73" s="4"/>
+      <c r="G73" s="4"/>
+      <c r="H73" s="4"/>
+      <c r="I73" s="4"/>
+    </row>
+    <row r="74" spans="1:9" ht="30" customHeight="1">
+      <c r="A74" t="inlineStr" s="32">
+        <is>
+          <t>Decision rule: use Solver output as evidence, then recommend only after checking client fit, scenario resilience, concentration, and the Phase 1 mandate.</t>
+        </is>
+      </c>
+      <c r="B74" s="32"/>
+      <c r="C74" s="32"/>
+      <c r="D74" s="32"/>
+      <c r="E74" s="32"/>
+      <c r="F74" s="32"/>
+      <c r="G74" s="32"/>
+      <c r="H74" s="32"/>
+      <c r="I74" s="32"/>
+    </row>
   </sheetData>
-  <mergeCells count="27">
+  <mergeCells count="56">
     <mergeCell ref="C53:H53"/>
     <mergeCell ref="C54:H54"/>
     <mergeCell ref="C46:H46"/>
@@ -2466,16 +2800,45 @@
     <mergeCell ref="A29:I29"/>
     <mergeCell ref="B30:D30"/>
     <mergeCell ref="A34:I34"/>
-    <mergeCell ref="E8:H8"/>
-    <mergeCell ref="E9:H9"/>
-    <mergeCell ref="E10:H10"/>
     <mergeCell ref="A13:I13"/>
     <mergeCell ref="A14:I14"/>
     <mergeCell ref="A2:I2"/>
     <mergeCell ref="A3:I3"/>
     <mergeCell ref="A4:I4"/>
     <mergeCell ref="A6:I6"/>
-    <mergeCell ref="E7:H7"/>
+    <mergeCell ref="E7:F7"/>
+    <mergeCell ref="G7:H7"/>
+    <mergeCell ref="E8:F8"/>
+    <mergeCell ref="G8:H8"/>
+    <mergeCell ref="E9:F9"/>
+    <mergeCell ref="G9:H9"/>
+    <mergeCell ref="E10:F10"/>
+    <mergeCell ref="G10:H10"/>
+    <mergeCell ref="A56:I56"/>
+    <mergeCell ref="A57:I57"/>
+    <mergeCell ref="B58:I58"/>
+    <mergeCell ref="B59:I59"/>
+    <mergeCell ref="B60:I60"/>
+    <mergeCell ref="B61:I61"/>
+    <mergeCell ref="B62:I62"/>
+    <mergeCell ref="B63:I63"/>
+    <mergeCell ref="B64:I64"/>
+    <mergeCell ref="B65:I65"/>
+    <mergeCell ref="A68:I68"/>
+    <mergeCell ref="A69:I69"/>
+    <mergeCell ref="C70:D70"/>
+    <mergeCell ref="E70:F70"/>
+    <mergeCell ref="G70:H70"/>
+    <mergeCell ref="C71:D71"/>
+    <mergeCell ref="E71:F71"/>
+    <mergeCell ref="G71:H71"/>
+    <mergeCell ref="C72:D72"/>
+    <mergeCell ref="E72:F72"/>
+    <mergeCell ref="G72:H72"/>
+    <mergeCell ref="C73:D73"/>
+    <mergeCell ref="E73:F73"/>
+    <mergeCell ref="G73:H73"/>
+    <mergeCell ref="A74:I74"/>
   </mergeCells>
   <conditionalFormatting sqref="F24:F26">
     <cfRule type="cellIs" dxfId="7" priority="2" operator="equal">
@@ -2504,14 +2867,16 @@
   <sheetPr>
     <tabColor rgb="FF8B1A1A"/>
   </sheetPr>
-  <dimension ref="A1:I69"/>
+  <dimension ref="A1:I74"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="2" customWidth="1"/>
-    <col min="2" max="2" width="26" customWidth="1"/>
-    <col min="3" max="5" width="18" customWidth="1"/>
-    <col min="6" max="8" width="20" customWidth="1"/>
-    <col min="9" max="9" width="2" customWidth="1"/>
+    <col min="2" max="2" width="22" customWidth="1"/>
+    <col min="3" max="4" width="14" customWidth="1"/>
+    <col min="5" max="5" width="18" customWidth="1"/>
+    <col min="6" max="6" width="13" customWidth="1"/>
+    <col min="7" max="8" width="18" customWidth="1"/>
+    <col min="9" max="9" width="27" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -2541,9 +2906,11 @@
       <c r="H3" s="8"/>
       <c r="I3" s="8"/>
     </row>
-    <row r="4" spans="1:9" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
-        <v>77</v>
+    <row r="4" spans="1:9" ht="38" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>⚠  BEAR CASE: Change only the returns, volatilities, or correlations justified by your downside economic story. Do not mechanically lower every return.</t>
+        </is>
       </c>
       <c r="B4" s="1"/>
       <c r="C4" s="1"/>
@@ -2556,8 +2923,10 @@
     </row>
     <row r="5" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="6" spans="1:9" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="6" t="s">
-        <v>26</v>
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>SECTION 1 — EXPECTATION BUILDER</t>
+        </is>
       </c>
       <c r="B6" s="6"/>
       <c r="C6" s="6"/>
@@ -2568,24 +2937,43 @@
       <c r="H6" s="6"/>
       <c r="I6" s="6"/>
     </row>
-    <row r="7" spans="1:9" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B7" s="16" t="s">
-        <v>27</v>
-      </c>
-      <c r="C7" s="16" t="s">
-        <v>28</v>
-      </c>
-      <c r="D7" s="16" t="s">
-        <v>29</v>
-      </c>
-      <c r="E7" s="5" t="s">
-        <v>30</v>
+    <row r="7" spans="1:9" ht="42" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B7" s="16" t="inlineStr">
+        <is>
+          <t>Asset Class</t>
+        </is>
+      </c>
+      <c r="C7" s="16" t="inlineStr">
+        <is>
+          <t>Expected Return
+E(R)</t>
+        </is>
+      </c>
+      <c r="D7" s="16" t="inlineStr">
+        <is>
+          <t>Volatility
+(σ)</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>Source + as-of date</t>
+        </is>
       </c>
       <c r="F7" s="5"/>
-      <c r="G7" s="5"/>
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>Downside rationale</t>
+        </is>
+      </c>
       <c r="H7" s="5"/>
-    </row>
-    <row r="8" spans="1:9" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I7" t="inlineStr" s="16">
+        <is>
+          <t>What changed from Base &amp; why</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" spans="1:9" ht="50" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B8" s="17" t="s">
         <v>31</v>
       </c>
@@ -2595,8 +2983,9 @@
       <c r="F8" s="4"/>
       <c r="G8" s="4"/>
       <c r="H8" s="4"/>
-    </row>
-    <row r="9" spans="1:9" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I8" s="4"/>
+    </row>
+    <row r="9" spans="1:9" ht="50" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B9" s="17" t="s">
         <v>32</v>
       </c>
@@ -2606,8 +2995,9 @@
       <c r="F9" s="4"/>
       <c r="G9" s="4"/>
       <c r="H9" s="4"/>
-    </row>
-    <row r="10" spans="1:9" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I9" s="4"/>
+    </row>
+    <row r="10" spans="1:9" ht="50" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B10" s="17" t="s">
         <v>33</v>
       </c>
@@ -2617,6 +3007,7 @@
       <c r="F10" s="4"/>
       <c r="G10" s="4"/>
       <c r="H10" s="4"/>
+      <c r="I10" s="4"/>
     </row>
     <row r="11" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="12" spans="1:9" ht="9.75" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -2633,9 +3024,11 @@
       <c r="H13" s="11"/>
       <c r="I13" s="11"/>
     </row>
-    <row r="14" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="12" t="s">
-        <v>78</v>
+    <row r="14" spans="1:9" ht="32" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="12" t="inlineStr">
+        <is>
+          <t>Change only correlations supported by the downside story and explain why. Do not force every correlation toward 1.0. Diagonal = 1.00.</t>
+        </is>
       </c>
       <c r="B14" s="12"/>
       <c r="C14" s="12"/>
@@ -2714,9 +3107,11 @@
       <c r="H21" s="11"/>
       <c r="I21" s="11"/>
     </row>
-    <row r="22" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="12" t="s">
-        <v>39</v>
+    <row r="22" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="12" t="inlineStr">
+        <is>
+          <t>Enter each client's starting weights, then run Solver one client at a time. Keep the Solver-supported weights only after completing the Section 6 usability checks.</t>
+        </is>
       </c>
       <c r="B22" s="12"/>
       <c r="C22" s="12"/>
@@ -2866,9 +3261,11 @@
       <c r="H34" s="11"/>
       <c r="I34" s="11"/>
     </row>
-    <row r="35" spans="1:9" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="12" t="s">
-        <v>54</v>
+    <row r="35" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="12" t="inlineStr">
+        <is>
+          <t>Use the Phase 1 IPS constraints. Portfolio σ is the active Solver risk limit; the drawdown tripwire remains a separate stress-test and recommendation check.</t>
+        </is>
       </c>
       <c r="B35" s="12"/>
       <c r="C35" s="12"/>
@@ -3087,22 +3484,269 @@
       <c r="H54" s="3"/>
     </row>
     <row r="55" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="56" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="57" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="58" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="59" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="60" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="61" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="62" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="63" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="64" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="65" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="56" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A56" t="inlineStr" s="11">
+        <is>
+          <t>SECTION 6 — SOLVER SETUP — RUN ONE CLIENT AT A TIME</t>
+        </is>
+      </c>
+      <c r="B56" s="11"/>
+      <c r="C56" s="11"/>
+      <c r="D56" s="11"/>
+      <c r="E56" s="11"/>
+      <c r="F56" s="11"/>
+      <c r="G56" s="11"/>
+      <c r="H56" s="11"/>
+      <c r="I56" s="11"/>
+    </row>
+    <row r="57" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A57" t="inlineStr" s="12">
+        <is>
+          <t>Use this checklist on the Bear Case sheet. Solver supports the recommendation; it does not decide whether the result fits the client.</t>
+        </is>
+      </c>
+      <c r="B57" s="12"/>
+      <c r="C57" s="12"/>
+      <c r="D57" s="12"/>
+      <c r="E57" s="12"/>
+      <c r="F57" s="12"/>
+      <c r="G57" s="12"/>
+      <c r="H57" s="12"/>
+      <c r="I57" s="12"/>
+    </row>
+    <row r="58" spans="1:9" ht="34" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B58" t="inlineStr" s="12">
+        <is>
+          <t>1. Understand the task — Solver searches the three asset-class weights for one client and scenario to maximize that row's Sharpe Ratio while respecting the listed constraints.</t>
+        </is>
+      </c>
+      <c r="C58" s="12"/>
+      <c r="D58" s="12"/>
+      <c r="E58" s="12"/>
+      <c r="F58" s="12"/>
+      <c r="G58" s="12"/>
+      <c r="H58" s="12"/>
+      <c r="I58" s="12"/>
+    </row>
+    <row r="59" spans="1:9" ht="34" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B59" t="inlineStr" s="12">
+        <is>
+          <t>2. Select the objective — Set I24, I25, or I26 to Max for Client 1, 2, or 3. Work on one client row at a time.</t>
+        </is>
+      </c>
+      <c r="C59" s="12"/>
+      <c r="D59" s="12"/>
+      <c r="E59" s="12"/>
+      <c r="F59" s="12"/>
+      <c r="G59" s="12"/>
+      <c r="H59" s="12"/>
+      <c r="I59" s="12"/>
+    </row>
+    <row r="60" spans="1:9" ht="34" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B60" t="inlineStr" s="12">
+        <is>
+          <t>3. Select changing cells — Use C24:E24, C25:E25, or C26:E26 for the same client row. These are the U.S. equity, fixed-income, and cash weights.</t>
+        </is>
+      </c>
+      <c r="C60" s="12"/>
+      <c r="D60" s="12"/>
+      <c r="E60" s="12"/>
+      <c r="F60" s="12"/>
+      <c r="G60" s="12"/>
+      <c r="H60" s="12"/>
+      <c r="I60" s="12"/>
+    </row>
+    <row r="61" spans="1:9" ht="42" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B61" t="inlineStr" s="32">
+        <is>
+          <t>4. Add the actual constraints — Matching row F = 1; matching row C:E ≥ 0; and H24 ≤ C37, H25 ≤ C38, or H26 ≤ C39. Drawdown in E37:E39 is not calculated by this model and is not a Solver constraint.</t>
+        </is>
+      </c>
+      <c r="C61" s="32"/>
+      <c r="D61" s="32"/>
+      <c r="E61" s="32"/>
+      <c r="F61" s="32"/>
+      <c r="G61" s="32"/>
+      <c r="H61" s="32"/>
+      <c r="I61" s="32"/>
+    </row>
+    <row r="62" spans="1:9" ht="34" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B62" t="inlineStr" s="12">
+        <is>
+          <t>5. Run Solver — Choose GRG Nonlinear, click Solve, and keep the Solver solution only if Solver reports a solution and the next checks pass.</t>
+        </is>
+      </c>
+      <c r="C62" s="12"/>
+      <c r="D62" s="12"/>
+      <c r="E62" s="12"/>
+      <c r="F62" s="12"/>
+      <c r="G62" s="12"/>
+      <c r="H62" s="12"/>
+      <c r="I62" s="12"/>
+    </row>
+    <row r="63" spans="1:9" ht="42" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B63" t="inlineStr" s="12">
+        <is>
+          <t>6. Confirm it is usable — Weights are nonnegative and total 100%; portfolio σ is within the matching Phase 1 limit; Status shows PASS; inputs use consistent percentage units; and the allocation is economically plausible for the client.</t>
+        </is>
+      </c>
+      <c r="C63" s="12"/>
+      <c r="D63" s="12"/>
+      <c r="E63" s="12"/>
+      <c r="F63" s="12"/>
+      <c r="G63" s="12"/>
+      <c r="H63" s="12"/>
+      <c r="I63" s="12"/>
+    </row>
+    <row r="64" spans="1:9" ht="42" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B64" t="inlineStr" s="32">
+        <is>
+          <t>7. If Solver is infeasible — Check the objective/changing/constraint cells all use the same client row, correlations are between –1 and 1, percentages were entered as percentages, and the IPS σ limit is entered. Do not relax an approved IPS limit to force a solution.</t>
+        </is>
+      </c>
+      <c r="C64" s="32"/>
+      <c r="D64" s="32"/>
+      <c r="E64" s="32"/>
+      <c r="F64" s="32"/>
+      <c r="G64" s="32"/>
+      <c r="H64" s="32"/>
+      <c r="I64" s="32"/>
+    </row>
+    <row r="65" ht="42" customHeight="1" x14ac:dyDescent="0.25" spans="1:9">
+      <c r="B65" t="inlineStr" s="32">
+        <is>
+          <t>8. If the allocation looks implausible — Recheck return, volatility, correlation, source/date, and starting weights. The Sharpe objective can concentrate a portfolio; use the stress test and client mandate before recommending it.</t>
+        </is>
+      </c>
+      <c r="C65" s="32"/>
+      <c r="D65" s="32"/>
+      <c r="E65" s="32"/>
+      <c r="F65" s="32"/>
+      <c r="G65" s="32"/>
+      <c r="H65" s="32"/>
+      <c r="I65" s="32"/>
+    </row>
     <row r="66" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="67" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="68" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="69" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="68" ht="24" customHeight="1" x14ac:dyDescent="0.25" spans="1:9">
+      <c r="A68" t="inlineStr" s="11">
+        <is>
+          <t>SECTION 7 — READ THE RESULT</t>
+        </is>
+      </c>
+      <c r="B68" s="11"/>
+      <c r="C68" s="11"/>
+      <c r="D68" s="11"/>
+      <c r="E68" s="11"/>
+      <c r="F68" s="11"/>
+      <c r="G68" s="11"/>
+      <c r="H68" s="11"/>
+      <c r="I68" s="11"/>
+    </row>
+    <row r="69" ht="30" customHeight="1" x14ac:dyDescent="0.25" spans="1:9">
+      <c r="A69" t="inlineStr" s="12">
+        <is>
+          <t>After Solver, interpret each client's Bear Case result against the starting allocation and Base Case. Keep answers concise and decision-focused.</t>
+        </is>
+      </c>
+      <c r="B69" s="12"/>
+      <c r="C69" s="12"/>
+      <c r="D69" s="12"/>
+      <c r="E69" s="12"/>
+      <c r="F69" s="12"/>
+      <c r="G69" s="12"/>
+      <c r="H69" s="12"/>
+      <c r="I69" s="12"/>
+    </row>
+    <row r="70" spans="1:9" ht="38" customHeight="1">
+      <c r="B70" t="inlineStr" s="16">
+        <is>
+          <t>Client</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr" s="16">
+        <is>
+          <t>Change from Base / starting allocation</t>
+        </is>
+      </c>
+      <c r="D70" s="16"/>
+      <c r="E70" t="inlineStr" s="16">
+        <is>
+          <t>Assumption or constraint driving it</t>
+        </is>
+      </c>
+      <c r="F70" s="16"/>
+      <c r="G70" t="inlineStr" s="16">
+        <is>
+          <t>Main trade-off</t>
+        </is>
+      </c>
+      <c r="H70" s="16"/>
+      <c r="I70" t="inlineStr" s="16">
+        <is>
+          <t>Revisit trigger</t>
+        </is>
+      </c>
+    </row>
+    <row r="71" spans="1:9" ht="52" customHeight="1">
+      <c r="B71" t="inlineStr" s="17">
+        <is>
+          <t>Client 1</t>
+        </is>
+      </c>
+      <c r="C71" s="4"/>
+      <c r="D71" s="4"/>
+      <c r="E71" s="4"/>
+      <c r="F71" s="4"/>
+      <c r="G71" s="4"/>
+      <c r="H71" s="4"/>
+      <c r="I71" s="4"/>
+    </row>
+    <row r="72" spans="1:9" ht="52" customHeight="1">
+      <c r="B72" t="inlineStr" s="17">
+        <is>
+          <t>Client 2</t>
+        </is>
+      </c>
+      <c r="C72" s="4"/>
+      <c r="D72" s="4"/>
+      <c r="E72" s="4"/>
+      <c r="F72" s="4"/>
+      <c r="G72" s="4"/>
+      <c r="H72" s="4"/>
+      <c r="I72" s="4"/>
+    </row>
+    <row r="73" spans="1:9" ht="52" customHeight="1">
+      <c r="B73" t="inlineStr" s="17">
+        <is>
+          <t>Client 3</t>
+        </is>
+      </c>
+      <c r="C73" s="4"/>
+      <c r="D73" s="4"/>
+      <c r="E73" s="4"/>
+      <c r="F73" s="4"/>
+      <c r="G73" s="4"/>
+      <c r="H73" s="4"/>
+      <c r="I73" s="4"/>
+    </row>
+    <row r="74" spans="1:9" ht="30" customHeight="1">
+      <c r="A74" t="inlineStr" s="32">
+        <is>
+          <t>Decision rule: use Solver output as evidence, then recommend only after checking client fit, scenario resilience, concentration, and the Phase 1 mandate.</t>
+        </is>
+      </c>
+      <c r="B74" s="32"/>
+      <c r="C74" s="32"/>
+      <c r="D74" s="32"/>
+      <c r="E74" s="32"/>
+      <c r="F74" s="32"/>
+      <c r="G74" s="32"/>
+      <c r="H74" s="32"/>
+      <c r="I74" s="32"/>
+    </row>
   </sheetData>
-  <mergeCells count="27">
+  <mergeCells count="56">
     <mergeCell ref="C53:H53"/>
     <mergeCell ref="C54:H54"/>
     <mergeCell ref="C46:H46"/>
@@ -3120,16 +3764,45 @@
     <mergeCell ref="A29:I29"/>
     <mergeCell ref="B30:D30"/>
     <mergeCell ref="A34:I34"/>
-    <mergeCell ref="E8:H8"/>
-    <mergeCell ref="E9:H9"/>
-    <mergeCell ref="E10:H10"/>
     <mergeCell ref="A13:I13"/>
     <mergeCell ref="A14:I14"/>
     <mergeCell ref="A2:I2"/>
     <mergeCell ref="A3:I3"/>
     <mergeCell ref="A4:I4"/>
     <mergeCell ref="A6:I6"/>
-    <mergeCell ref="E7:H7"/>
+    <mergeCell ref="E7:F7"/>
+    <mergeCell ref="G7:H7"/>
+    <mergeCell ref="E8:F8"/>
+    <mergeCell ref="G8:H8"/>
+    <mergeCell ref="E9:F9"/>
+    <mergeCell ref="G9:H9"/>
+    <mergeCell ref="E10:F10"/>
+    <mergeCell ref="G10:H10"/>
+    <mergeCell ref="A56:I56"/>
+    <mergeCell ref="A57:I57"/>
+    <mergeCell ref="B58:I58"/>
+    <mergeCell ref="B59:I59"/>
+    <mergeCell ref="B60:I60"/>
+    <mergeCell ref="B61:I61"/>
+    <mergeCell ref="B62:I62"/>
+    <mergeCell ref="B63:I63"/>
+    <mergeCell ref="B64:I64"/>
+    <mergeCell ref="B65:I65"/>
+    <mergeCell ref="A68:I68"/>
+    <mergeCell ref="A69:I69"/>
+    <mergeCell ref="C70:D70"/>
+    <mergeCell ref="E70:F70"/>
+    <mergeCell ref="G70:H70"/>
+    <mergeCell ref="C71:D71"/>
+    <mergeCell ref="E71:F71"/>
+    <mergeCell ref="G71:H71"/>
+    <mergeCell ref="C72:D72"/>
+    <mergeCell ref="E72:F72"/>
+    <mergeCell ref="G72:H72"/>
+    <mergeCell ref="C73:D73"/>
+    <mergeCell ref="E73:F73"/>
+    <mergeCell ref="G73:H73"/>
+    <mergeCell ref="A74:I74"/>
   </mergeCells>
   <conditionalFormatting sqref="F24:F26">
     <cfRule type="cellIs" dxfId="3" priority="2" operator="equal">

</xml_diff>